<commit_message>
Update Uji Testing CRUD
</commit_message>
<xml_diff>
--- a/backup/matakuliah_backup.xlsx
+++ b/backup/matakuliah_backup.xlsx
@@ -431,12 +431,12 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Kode</t>
+          <t>Kode MK</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Matakuliah</t>
+          <t>Nama Matakuliah</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -446,12 +446,12 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Smt</t>
+          <t>Semester</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Prodi</t>
+          <t>Program Studi</t>
         </is>
       </c>
     </row>

</xml_diff>